<commit_message>
feat: bilingual LLM output, similar perfumes, db en columns, weather i18n
Backend:
- Agent2 parallel zh/en DeepSeek prompts with max_tokens=1200
- New SimilarPerfume schema + similar_perfumes list (2-3 items, bilingual)
- FormulaNote.name_en for consumer-friendly English ingredient names
- FinalOutput adds scent_description_en + selection_rationale_en
- translate_ingredients.py one-shot script populates English columns in ingredients.xlsx
- Enhanced exception logging in LLM call paths

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/database/data/ingredients.xlsx
+++ b/backend/database/data/ingredients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,6 +484,26 @@
           <t>in_stock</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>function_en</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>description_en</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>usage_en</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>caution_level_en</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -536,6 +556,26 @@
       </c>
       <c r="K2" t="b">
         <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Fresh top note combination</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Classic citrus top note</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Cologne/tea/refreshing</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -590,6 +630,26 @@
       <c r="K3" t="b">
         <v>1</v>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Transparent woody</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Transparent woody diffusion</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Woody, airy, diffusion</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -643,6 +703,26 @@
       <c r="K4" t="b">
         <v>1</v>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Floral connector</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Fresh floral connector</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>White floral, citrus, soapy</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -696,6 +776,26 @@
       <c r="K5" t="b">
         <v>1</v>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Airy white floral</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>White floral airy core</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>White floral, green, aquatic</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -749,6 +849,26 @@
       <c r="K6" t="b">
         <v>1</v>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Green leaf</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Green leaf, high impact</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Grass, leaf, morning dew</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -802,6 +922,26 @@
       <c r="K7" t="b">
         <v>1</v>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Clean musk</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Clean lasting skeleton</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Daily chemical, lasting, base</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -855,6 +995,26 @@
       <c r="K8" t="b">
         <v>1</v>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Sweet warm resin</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Sweet warm resin fixative</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Vanilla, oriental, amber</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -908,6 +1068,26 @@
       <c r="K9" t="b">
         <v>1</v>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Floral main body</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Rose/floral main body</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Rose, bouquet, watery floral</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -961,6 +1141,26 @@
       <c r="K10" t="b">
         <v>1</v>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Melon aquatic</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Aquatic melon, high impact</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Melon, watermelon, clear water</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1014,6 +1214,26 @@
       <c r="K11" t="b">
         <v>1</v>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Peach milky fruity</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Peach milky fruity</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Peach, apricot, milky</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1067,6 +1287,26 @@
       <c r="K12" t="b">
         <v>1</v>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Woody amber</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Woody amber velvety</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Woody, velvety, warmth</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1120,6 +1360,26 @@
       <c r="K13" t="b">
         <v>1</v>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Marine aquatic</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Seawater/ozone</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Sea breeze, saltwater, watermelon rind</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1173,6 +1433,26 @@
       <c r="K14" t="b">
         <v>1</v>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Violet</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Violet/powdery</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Powdery, woody floral</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1226,6 +1506,26 @@
       <c r="K15" t="b">
         <v>1</v>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Sugar cotton candy</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Sugar enhancement</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Caramel sugar, dessert</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1279,6 +1579,26 @@
       <c r="K16" t="b">
         <v>1</v>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Soft white musk</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Soft white musk</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Skin-like, soft drydown</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1332,6 +1652,26 @@
       <c r="K17" t="b">
         <v>1</v>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Advanced accent</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Spicy carnation</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Leather, white floral animalic, spicy</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1385,6 +1725,26 @@
       <c r="K18" t="b">
         <v>1</v>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Woody skeleton</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Woody skeleton</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Dry wood, pencil wood, tea wood</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1438,6 +1798,26 @@
       <c r="K19" t="b">
         <v>1</v>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>White floral fruity</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>White floral fruity</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Jasmine, banana white floral, fruity</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1491,6 +1871,26 @@
       <c r="K20" t="b">
         <v>1</v>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Fresh top note combination</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Bright lemon top note</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Cologne/tea/refreshing</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1544,6 +1944,26 @@
       <c r="K21" t="b">
         <v>1</v>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Lemon peel</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Lemon peel sharpness</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Fresh lemon, sharpness</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1597,6 +2017,26 @@
       <c r="K22" t="b">
         <v>1</v>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Advanced accent</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Tar leather smoky</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Leather, white floral animalic, spicy</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1650,6 +2090,26 @@
       <c r="K23" t="b">
         <v>1</v>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Vanilla main body</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Vanilla sweet main body</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Vanilla, milky sweet, gourmand</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1703,6 +2163,26 @@
       <c r="K24" t="b">
         <v>1</v>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Warm sweet bean</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Tonka bean/warm sweet</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Tonka bean, vanilla, tobacco</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1756,6 +2236,26 @@
       <c r="K25" t="b">
         <v>1</v>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Violet rose</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Violet/rose enhancement</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Rose violet, powdery</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1808,6 +2308,26 @@
       </c>
       <c r="K26" t="b">
         <v>1</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Woody fixation</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Woody earthy fixation</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Patchouli, earthy, stable</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1846,6 +2366,14 @@
       <c r="K27" t="b">
         <v>1</v>
       </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Crisp fruity top note</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1899,6 +2427,26 @@
       <c r="K28" t="b">
         <v>1</v>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Fixative/solvent</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Fixative/solvent auxiliary</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Fixative, dissolve resin</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1952,6 +2500,26 @@
       <c r="K29" t="b">
         <v>1</v>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Clean musk</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Metallic clean musk</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Modern clean, metallic</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2004,6 +2572,26 @@
       </c>
       <c r="K30" t="b">
         <v>1</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Soft musk</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Soft macrocyclic musk</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Gentle milky white, comfortable lasting</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2042,6 +2630,14 @@
       <c r="K31" t="b">
         <v>1</v>
       </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Aromatic herbal fresh</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2095,6 +2691,26 @@
       <c r="K32" t="b">
         <v>1</v>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Advanced accent</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>White floral animalic, dilute first</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Leather, white floral animalic, spicy</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2147,6 +2763,26 @@
       </c>
       <c r="K33" t="b">
         <v>1</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Spicy sweet resin</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Sweet spicy resin base</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Oriental, resin, leather</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -2185,6 +2821,14 @@
       <c r="K34" t="b">
         <v>1</v>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Can directly create tea theme</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2238,6 +2882,26 @@
       <c r="K35" t="b">
         <v>1</v>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Berry floral sweet</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Berry floral sweet connector</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Berry, rose-like</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2291,6 +2955,26 @@
       <c r="K36" t="b">
         <v>1</v>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Caramel jam</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Caramel jam sweetness</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Syrup, jam, caramel</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2343,6 +3027,26 @@
       </c>
       <c r="K37" t="b">
         <v>1</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Round musk</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Soft round white musk</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Soapy, clean, finish</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -2381,6 +3085,14 @@
       <c r="K38" t="b">
         <v>1</v>
       </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Powdery iris shortcut</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2433,6 +3145,26 @@
       </c>
       <c r="K39" t="b">
         <v>1</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Brighten white floral</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Brighter floral airy</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Brighter jasmine-like</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>